<commit_message>
new data 5 mai 2025
</commit_message>
<xml_diff>
--- a/data/spike.xlsx
+++ b/data/spike.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\phbro\Desktop\DOCUMENTS\ActuRank\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFC6FA50-B278-46E4-BB28-CE0C6C8B6473}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA4AC837-1345-4EE9-B6E5-503C67BC7EEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1068" yWindow="-108" windowWidth="22080" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="516" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="646" uniqueCount="66">
   <si>
     <t>players</t>
   </si>
@@ -231,6 +231,9 @@
   </si>
   <si>
     <t>31/10/2024</t>
+  </si>
+  <si>
+    <t>05/05/2025</t>
   </si>
 </sst>
 </file>
@@ -3367,7 +3370,7 @@
         <v>11</v>
       </c>
       <c r="E68" s="1">
-        <f t="shared" ref="E68:E94" si="2">IF(F68&gt;G68,1,0)</f>
+        <f t="shared" ref="E68:E120" si="2">IF(F68&gt;G68,1,0)</f>
         <v>1</v>
       </c>
       <c r="F68" s="5">
@@ -3384,7 +3387,7 @@
       </c>
       <c r="J68" s="1"/>
       <c r="K68" s="9" t="str">
-        <f t="shared" ref="K68:K94" si="3">IF(OR(OR(AND(OR(A68=B68,A68=C68,A68=D68,B68=C68,B68=D68,C68=D68),OR(A68&lt;&gt;"",D68&lt;&gt;"")),H68&gt;MAX(F68:G68),B68=C68),OR(AND(ISBLANK(A68)=FALSE,ISNA(VLOOKUP(A68,$M$3:$O$27,1,FALSE))),ISNA(VLOOKUP(B68,$M$3:$O$27,1,FALSE)),ISNA(VLOOKUP(C68,$M$3:$O$27,1,FALSE)),AND(ISBLANK(D68)=FALSE,ISNA(VLOOKUP(D68,$M$3:$O$27,1,FALSE))),OR(COUNTBLANK(A68:D68)=1,COUNTBLANK(A68:D68)=3))),"ERREUR","")</f>
+        <f t="shared" ref="K68:K120" si="3">IF(OR(OR(AND(OR(A68=B68,A68=C68,A68=D68,B68=C68,B68=D68,C68=D68),OR(A68&lt;&gt;"",D68&lt;&gt;"")),H68&gt;MAX(F68:G68),B68=C68),OR(AND(ISBLANK(A68)=FALSE,ISNA(VLOOKUP(A68,$M$3:$O$27,1,FALSE))),ISNA(VLOOKUP(B68,$M$3:$O$27,1,FALSE)),ISNA(VLOOKUP(C68,$M$3:$O$27,1,FALSE)),AND(ISBLANK(D68)=FALSE,ISNA(VLOOKUP(D68,$M$3:$O$27,1,FALSE))),OR(COUNTBLANK(A68:D68)=1,COUNTBLANK(A68:D68)=3))),"ERREUR","")</f>
         <v/>
       </c>
       <c r="L68" s="1"/>
@@ -4407,442 +4410,1014 @@
       <c r="O94" s="1"/>
     </row>
     <row r="95" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A95" s="6"/>
-      <c r="B95" s="6"/>
-      <c r="C95" s="7"/>
-      <c r="D95" s="7"/>
-      <c r="E95" s="1"/>
-      <c r="F95" s="5"/>
-      <c r="G95" s="5"/>
-      <c r="H95" s="1"/>
-      <c r="I95" s="1"/>
+      <c r="A95" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B95" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C95" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="D95" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E95" s="1">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="F95" s="5">
+        <v>8</v>
+      </c>
+      <c r="G95" s="5">
+        <v>6</v>
+      </c>
+      <c r="H95" s="1">
+        <v>7</v>
+      </c>
+      <c r="I95" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="J95" s="1"/>
-      <c r="K95" s="9"/>
+      <c r="K95" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="L95" s="1"/>
       <c r="M95" s="1"/>
       <c r="N95" s="1"/>
       <c r="O95" s="1"/>
     </row>
     <row r="96" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A96" s="6"/>
-      <c r="B96" s="6"/>
-      <c r="C96" s="7"/>
-      <c r="D96" s="7"/>
-      <c r="E96" s="1"/>
-      <c r="F96" s="5"/>
-      <c r="G96" s="5"/>
-      <c r="H96" s="1"/>
-      <c r="I96" s="1"/>
+      <c r="A96" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B96" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C96" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D96" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E96" s="1">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="F96" s="5">
+        <v>8</v>
+      </c>
+      <c r="G96" s="5">
+        <v>6</v>
+      </c>
+      <c r="H96" s="1">
+        <v>7</v>
+      </c>
+      <c r="I96" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="J96" s="1"/>
-      <c r="K96" s="9"/>
+      <c r="K96" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="L96" s="1"/>
       <c r="M96" s="1"/>
       <c r="N96" s="1"/>
       <c r="O96" s="1"/>
     </row>
     <row r="97" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A97" s="6"/>
-      <c r="B97" s="6"/>
-      <c r="C97" s="7"/>
-      <c r="D97" s="7"/>
-      <c r="E97" s="1"/>
-      <c r="F97" s="5"/>
-      <c r="G97" s="5"/>
-      <c r="H97" s="1"/>
-      <c r="I97" s="1"/>
+      <c r="A97" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B97" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C97" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="D97" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E97" s="1">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="F97" s="5">
+        <v>7</v>
+      </c>
+      <c r="G97" s="5">
+        <v>5</v>
+      </c>
+      <c r="H97" s="1">
+        <v>7</v>
+      </c>
+      <c r="I97" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="J97" s="1"/>
-      <c r="K97" s="9"/>
+      <c r="K97" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="L97" s="1"/>
       <c r="M97" s="1"/>
       <c r="N97" s="1"/>
       <c r="O97" s="1"/>
     </row>
     <row r="98" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A98" s="6"/>
-      <c r="B98" s="6"/>
-      <c r="C98" s="7"/>
-      <c r="D98" s="7"/>
-      <c r="E98" s="1"/>
-      <c r="F98" s="5"/>
-      <c r="G98" s="5"/>
-      <c r="H98" s="1"/>
-      <c r="I98" s="1"/>
+      <c r="A98" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B98" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C98" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D98" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E98" s="1">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="F98" s="5">
+        <v>7</v>
+      </c>
+      <c r="G98" s="5">
+        <v>0</v>
+      </c>
+      <c r="H98" s="1">
+        <v>7</v>
+      </c>
+      <c r="I98" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="J98" s="1"/>
-      <c r="K98" s="9"/>
+      <c r="K98" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="L98" s="1"/>
       <c r="M98" s="1"/>
       <c r="N98" s="1"/>
       <c r="O98" s="1"/>
     </row>
     <row r="99" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A99" s="6"/>
-      <c r="B99" s="6"/>
-      <c r="C99" s="7"/>
-      <c r="D99" s="7"/>
-      <c r="E99" s="1"/>
-      <c r="F99" s="5"/>
-      <c r="G99" s="5"/>
-      <c r="H99" s="1"/>
-      <c r="I99" s="1"/>
+      <c r="A99" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B99" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C99" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="D99" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E99" s="1">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="F99" s="5">
+        <v>7</v>
+      </c>
+      <c r="G99" s="5">
+        <v>2</v>
+      </c>
+      <c r="H99" s="1">
+        <v>7</v>
+      </c>
+      <c r="I99" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="J99" s="1"/>
-      <c r="K99" s="9"/>
+      <c r="K99" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="L99" s="1"/>
       <c r="M99" s="1"/>
       <c r="N99" s="1"/>
       <c r="O99" s="1"/>
     </row>
     <row r="100" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A100" s="6"/>
-      <c r="B100" s="6"/>
-      <c r="C100" s="7"/>
-      <c r="D100" s="7"/>
-      <c r="E100" s="1"/>
-      <c r="F100" s="5"/>
-      <c r="G100" s="5"/>
-      <c r="H100" s="1"/>
-      <c r="I100" s="1"/>
+      <c r="A100" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B100" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C100" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D100" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E100" s="1">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="F100" s="5">
+        <v>7</v>
+      </c>
+      <c r="G100" s="5">
+        <v>5</v>
+      </c>
+      <c r="H100" s="1">
+        <v>7</v>
+      </c>
+      <c r="I100" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="J100" s="1"/>
-      <c r="K100" s="9"/>
+      <c r="K100" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="L100" s="1"/>
       <c r="M100" s="1"/>
       <c r="N100" s="1"/>
       <c r="O100" s="1"/>
     </row>
     <row r="101" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A101" s="6"/>
-      <c r="B101" s="6"/>
-      <c r="C101" s="7"/>
-      <c r="D101" s="7"/>
-      <c r="E101" s="1"/>
-      <c r="F101" s="5"/>
-      <c r="G101" s="5"/>
-      <c r="H101" s="1"/>
-      <c r="I101" s="1"/>
+      <c r="A101" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B101" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C101" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="D101" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E101" s="1">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="F101" s="5">
+        <v>7</v>
+      </c>
+      <c r="G101" s="5">
+        <v>4</v>
+      </c>
+      <c r="H101" s="1">
+        <v>7</v>
+      </c>
+      <c r="I101" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="J101" s="1"/>
-      <c r="K101" s="9"/>
+      <c r="K101" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="L101" s="1"/>
       <c r="M101" s="1"/>
       <c r="N101" s="1"/>
       <c r="O101" s="1"/>
     </row>
     <row r="102" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A102" s="6"/>
-      <c r="B102" s="6"/>
-      <c r="C102" s="7"/>
-      <c r="D102" s="7"/>
-      <c r="E102" s="1"/>
-      <c r="F102" s="5"/>
-      <c r="G102" s="5"/>
-      <c r="H102" s="1"/>
-      <c r="I102" s="1"/>
+      <c r="A102" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B102" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C102" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D102" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E102" s="1">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="F102" s="5">
+        <v>7</v>
+      </c>
+      <c r="G102" s="5">
+        <v>4</v>
+      </c>
+      <c r="H102" s="1">
+        <v>7</v>
+      </c>
+      <c r="I102" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="J102" s="1"/>
-      <c r="K102" s="9"/>
+      <c r="K102" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="L102" s="1"/>
       <c r="M102" s="1"/>
       <c r="N102" s="1"/>
       <c r="O102" s="1"/>
     </row>
     <row r="103" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A103" s="6"/>
-      <c r="B103" s="6"/>
-      <c r="C103" s="7"/>
-      <c r="D103" s="7"/>
-      <c r="E103" s="1"/>
-      <c r="F103" s="5"/>
-      <c r="G103" s="5"/>
-      <c r="H103" s="1"/>
-      <c r="I103" s="1"/>
+      <c r="A103" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B103" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C103" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="D103" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E103" s="1">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="F103" s="5">
+        <v>7</v>
+      </c>
+      <c r="G103" s="5">
+        <v>4</v>
+      </c>
+      <c r="H103" s="1">
+        <v>7</v>
+      </c>
+      <c r="I103" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="J103" s="1"/>
-      <c r="K103" s="9"/>
+      <c r="K103" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="L103" s="1"/>
       <c r="M103" s="1"/>
       <c r="N103" s="1"/>
       <c r="O103" s="1"/>
     </row>
     <row r="104" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A104" s="6"/>
-      <c r="B104" s="6"/>
-      <c r="C104" s="7"/>
-      <c r="D104" s="7"/>
-      <c r="E104" s="1"/>
-      <c r="F104" s="5"/>
-      <c r="G104" s="5"/>
-      <c r="H104" s="1"/>
-      <c r="I104" s="1"/>
+      <c r="A104" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B104" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C104" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D104" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E104" s="1">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="F104" s="5">
+        <v>7</v>
+      </c>
+      <c r="G104" s="5">
+        <v>4</v>
+      </c>
+      <c r="H104" s="1">
+        <v>7</v>
+      </c>
+      <c r="I104" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="J104" s="1"/>
-      <c r="K104" s="9"/>
+      <c r="K104" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="L104" s="1"/>
       <c r="M104" s="1"/>
       <c r="N104" s="1"/>
       <c r="O104" s="1"/>
     </row>
     <row r="105" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A105" s="6"/>
-      <c r="B105" s="6"/>
-      <c r="C105" s="7"/>
-      <c r="D105" s="7"/>
-      <c r="E105" s="1"/>
-      <c r="F105" s="5"/>
-      <c r="G105" s="5"/>
-      <c r="H105" s="1"/>
-      <c r="I105" s="1"/>
+      <c r="A105" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B105" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C105" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D105" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="E105" s="1">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="F105" s="5">
+        <v>7</v>
+      </c>
+      <c r="G105" s="5">
+        <v>0</v>
+      </c>
+      <c r="H105" s="1">
+        <v>7</v>
+      </c>
+      <c r="I105" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="J105" s="1"/>
-      <c r="K105" s="9"/>
+      <c r="K105" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="L105" s="1"/>
       <c r="M105" s="1"/>
       <c r="N105" s="1"/>
       <c r="O105" s="1"/>
     </row>
     <row r="106" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A106" s="6"/>
-      <c r="B106" s="6"/>
-      <c r="C106" s="7"/>
-      <c r="D106" s="7"/>
-      <c r="E106" s="1"/>
-      <c r="F106" s="5"/>
-      <c r="G106" s="5"/>
-      <c r="H106" s="1"/>
-      <c r="I106" s="1"/>
+      <c r="A106" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B106" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C106" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D106" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E106" s="1">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="F106" s="5">
+        <v>7</v>
+      </c>
+      <c r="G106" s="5">
+        <v>2</v>
+      </c>
+      <c r="H106" s="1">
+        <v>7</v>
+      </c>
+      <c r="I106" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="J106" s="1"/>
-      <c r="K106" s="9"/>
+      <c r="K106" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="L106" s="1"/>
       <c r="M106" s="1"/>
       <c r="N106" s="1"/>
       <c r="O106" s="1"/>
     </row>
     <row r="107" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A107" s="6"/>
-      <c r="B107" s="6"/>
-      <c r="C107" s="7"/>
-      <c r="D107" s="7"/>
-      <c r="E107" s="1"/>
-      <c r="F107" s="5"/>
-      <c r="G107" s="5"/>
-      <c r="H107" s="1"/>
-      <c r="I107" s="1"/>
+      <c r="A107" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B107" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C107" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="D107" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E107" s="1">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="F107" s="5">
+        <v>7</v>
+      </c>
+      <c r="G107" s="5">
+        <v>3</v>
+      </c>
+      <c r="H107" s="1">
+        <v>7</v>
+      </c>
+      <c r="I107" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="J107" s="1"/>
-      <c r="K107" s="9"/>
+      <c r="K107" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="L107" s="1"/>
       <c r="M107" s="1"/>
       <c r="N107" s="1"/>
       <c r="O107" s="1"/>
     </row>
     <row r="108" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A108" s="6"/>
-      <c r="B108" s="6"/>
-      <c r="C108" s="7"/>
-      <c r="D108" s="7"/>
-      <c r="E108" s="1"/>
-      <c r="F108" s="5"/>
-      <c r="G108" s="5"/>
-      <c r="H108" s="1"/>
-      <c r="I108" s="1"/>
+      <c r="A108" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B108" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C108" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="D108" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E108" s="1">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="F108" s="5">
+        <v>7</v>
+      </c>
+      <c r="G108" s="5">
+        <v>4</v>
+      </c>
+      <c r="H108" s="1">
+        <v>7</v>
+      </c>
+      <c r="I108" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="J108" s="1"/>
-      <c r="K108" s="9"/>
+      <c r="K108" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="L108" s="1"/>
       <c r="M108" s="1"/>
       <c r="N108" s="1"/>
       <c r="O108" s="1"/>
     </row>
     <row r="109" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A109" s="6"/>
-      <c r="B109" s="6"/>
-      <c r="C109" s="7"/>
-      <c r="D109" s="7"/>
-      <c r="E109" s="1"/>
-      <c r="F109" s="5"/>
-      <c r="G109" s="5"/>
-      <c r="H109" s="1"/>
-      <c r="I109" s="1"/>
+      <c r="A109" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B109" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C109" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D109" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E109" s="1">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="F109" s="5">
+        <v>7</v>
+      </c>
+      <c r="G109" s="5">
+        <v>4</v>
+      </c>
+      <c r="H109" s="1">
+        <v>7</v>
+      </c>
+      <c r="I109" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="J109" s="1"/>
-      <c r="K109" s="9"/>
+      <c r="K109" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="L109" s="1"/>
       <c r="M109" s="1"/>
       <c r="N109" s="1"/>
       <c r="O109" s="1"/>
     </row>
     <row r="110" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A110" s="6"/>
-      <c r="B110" s="6"/>
-      <c r="C110" s="7"/>
-      <c r="D110" s="7"/>
-      <c r="E110" s="1"/>
-      <c r="F110" s="5"/>
-      <c r="G110" s="5"/>
-      <c r="H110" s="1"/>
-      <c r="I110" s="1"/>
+      <c r="A110" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B110" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C110" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="D110" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E110" s="1">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="F110" s="5">
+        <v>7</v>
+      </c>
+      <c r="G110" s="5">
+        <v>2</v>
+      </c>
+      <c r="H110" s="1">
+        <v>7</v>
+      </c>
+      <c r="I110" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="J110" s="1"/>
-      <c r="K110" s="9"/>
+      <c r="K110" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="L110" s="1"/>
       <c r="M110" s="1"/>
       <c r="N110" s="1"/>
       <c r="O110" s="1"/>
     </row>
     <row r="111" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A111" s="6"/>
-      <c r="B111" s="6"/>
-      <c r="C111" s="7"/>
-      <c r="D111" s="7"/>
-      <c r="E111" s="1"/>
-      <c r="F111" s="5"/>
-      <c r="G111" s="5"/>
-      <c r="H111" s="1"/>
-      <c r="I111" s="1"/>
+      <c r="A111" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B111" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C111" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D111" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E111" s="1">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="F111" s="5">
+        <v>7</v>
+      </c>
+      <c r="G111" s="5">
+        <v>3</v>
+      </c>
+      <c r="H111" s="1">
+        <v>7</v>
+      </c>
+      <c r="I111" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="J111" s="1"/>
-      <c r="K111" s="9"/>
+      <c r="K111" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="L111" s="1"/>
       <c r="M111" s="1"/>
       <c r="N111" s="1"/>
       <c r="O111" s="1"/>
     </row>
     <row r="112" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A112" s="6"/>
-      <c r="B112" s="6"/>
-      <c r="C112" s="7"/>
-      <c r="D112" s="7"/>
-      <c r="E112" s="1"/>
-      <c r="F112" s="5"/>
-      <c r="G112" s="5"/>
-      <c r="H112" s="1"/>
-      <c r="I112" s="1"/>
+      <c r="A112" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B112" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C112" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D112" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="E112" s="1">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="F112" s="5">
+        <v>7</v>
+      </c>
+      <c r="G112" s="5">
+        <v>3</v>
+      </c>
+      <c r="H112" s="1">
+        <v>7</v>
+      </c>
+      <c r="I112" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="J112" s="1"/>
-      <c r="K112" s="9"/>
+      <c r="K112" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="L112" s="1"/>
       <c r="M112" s="1"/>
       <c r="N112" s="1"/>
       <c r="O112" s="1"/>
     </row>
     <row r="113" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A113" s="6"/>
-      <c r="B113" s="6"/>
-      <c r="C113" s="7"/>
-      <c r="D113" s="7"/>
-      <c r="E113" s="1"/>
-      <c r="F113" s="5"/>
-      <c r="G113" s="5"/>
-      <c r="H113" s="1"/>
-      <c r="I113" s="1"/>
+      <c r="A113" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B113" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C113" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D113" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E113" s="1">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="F113" s="5">
+        <v>7</v>
+      </c>
+      <c r="G113" s="5">
+        <v>5</v>
+      </c>
+      <c r="H113" s="1">
+        <v>7</v>
+      </c>
+      <c r="I113" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="J113" s="1"/>
-      <c r="K113" s="9"/>
+      <c r="K113" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="L113" s="1"/>
       <c r="M113" s="1"/>
       <c r="N113" s="1"/>
       <c r="O113" s="1"/>
     </row>
     <row r="114" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A114" s="6"/>
-      <c r="B114" s="6"/>
-      <c r="C114" s="7"/>
-      <c r="D114" s="7"/>
-      <c r="E114" s="1"/>
-      <c r="F114" s="5"/>
-      <c r="G114" s="5"/>
-      <c r="H114" s="1"/>
-      <c r="I114" s="1"/>
+      <c r="A114" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B114" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C114" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D114" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E114" s="1">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="F114" s="5">
+        <v>7</v>
+      </c>
+      <c r="G114" s="5">
+        <v>3</v>
+      </c>
+      <c r="H114" s="1">
+        <v>7</v>
+      </c>
+      <c r="I114" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="J114" s="1"/>
-      <c r="K114" s="9"/>
+      <c r="K114" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="L114" s="1"/>
       <c r="M114" s="1"/>
       <c r="N114" s="1"/>
       <c r="O114" s="1"/>
     </row>
     <row r="115" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A115" s="6"/>
-      <c r="B115" s="6"/>
-      <c r="C115" s="7"/>
-      <c r="D115" s="7"/>
-      <c r="E115" s="1"/>
-      <c r="F115" s="5"/>
-      <c r="G115" s="5"/>
-      <c r="H115" s="1"/>
-      <c r="I115" s="1"/>
+      <c r="A115" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B115" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C115" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D115" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="E115" s="1">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="F115" s="5">
+        <v>7</v>
+      </c>
+      <c r="G115" s="5">
+        <v>4</v>
+      </c>
+      <c r="H115" s="1">
+        <v>7</v>
+      </c>
+      <c r="I115" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="J115" s="1"/>
-      <c r="K115" s="9"/>
+      <c r="K115" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="L115" s="1"/>
       <c r="M115" s="1"/>
       <c r="N115" s="1"/>
       <c r="O115" s="1"/>
     </row>
     <row r="116" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A116" s="6"/>
-      <c r="B116" s="6"/>
-      <c r="C116" s="7"/>
-      <c r="D116" s="7"/>
-      <c r="E116" s="1"/>
-      <c r="F116" s="5"/>
-      <c r="G116" s="5"/>
-      <c r="H116" s="1"/>
-      <c r="I116" s="1"/>
+      <c r="A116" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B116" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C116" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D116" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E116" s="1">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="F116" s="5">
+        <v>7</v>
+      </c>
+      <c r="G116" s="5">
+        <v>2</v>
+      </c>
+      <c r="H116" s="1">
+        <v>7</v>
+      </c>
+      <c r="I116" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="J116" s="1"/>
-      <c r="K116" s="9"/>
+      <c r="K116" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="L116" s="1"/>
       <c r="M116" s="1"/>
       <c r="N116" s="1"/>
       <c r="O116" s="1"/>
     </row>
     <row r="117" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A117" s="6"/>
-      <c r="B117" s="6"/>
-      <c r="C117" s="7"/>
-      <c r="D117" s="7"/>
-      <c r="E117" s="1"/>
-      <c r="F117" s="5"/>
-      <c r="G117" s="5"/>
-      <c r="H117" s="1"/>
-      <c r="I117" s="1"/>
+      <c r="A117" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B117" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C117" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D117" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E117" s="1">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="F117" s="5">
+        <v>7</v>
+      </c>
+      <c r="G117" s="5">
+        <v>4</v>
+      </c>
+      <c r="H117" s="1">
+        <v>7</v>
+      </c>
+      <c r="I117" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="J117" s="1"/>
-      <c r="K117" s="9"/>
+      <c r="K117" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="L117" s="1"/>
       <c r="M117" s="1"/>
       <c r="N117" s="1"/>
       <c r="O117" s="1"/>
     </row>
     <row r="118" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A118" s="6"/>
-      <c r="B118" s="6"/>
-      <c r="C118" s="7"/>
-      <c r="D118" s="7"/>
-      <c r="E118" s="1"/>
-      <c r="F118" s="5"/>
-      <c r="G118" s="5"/>
-      <c r="H118" s="1"/>
-      <c r="I118" s="1"/>
+      <c r="A118" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B118" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C118" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D118" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="E118" s="1">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="F118" s="5">
+        <v>7</v>
+      </c>
+      <c r="G118" s="5">
+        <v>3</v>
+      </c>
+      <c r="H118" s="1">
+        <v>7</v>
+      </c>
+      <c r="I118" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="J118" s="1"/>
-      <c r="K118" s="9"/>
+      <c r="K118" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="L118" s="1"/>
       <c r="M118" s="1"/>
       <c r="N118" s="1"/>
       <c r="O118" s="1"/>
     </row>
     <row r="119" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A119" s="6"/>
-      <c r="B119" s="6"/>
-      <c r="C119" s="7"/>
-      <c r="D119" s="7"/>
-      <c r="E119" s="1"/>
-      <c r="F119" s="5"/>
-      <c r="G119" s="5"/>
-      <c r="H119" s="1"/>
-      <c r="I119" s="1"/>
+      <c r="A119" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B119" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C119" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D119" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E119" s="1">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="F119" s="5">
+        <v>7</v>
+      </c>
+      <c r="G119" s="5">
+        <v>2</v>
+      </c>
+      <c r="H119" s="1">
+        <v>7</v>
+      </c>
+      <c r="I119" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="J119" s="1"/>
-      <c r="K119" s="9"/>
+      <c r="K119" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="L119" s="1"/>
       <c r="M119" s="1"/>
       <c r="N119" s="1"/>
       <c r="O119" s="1"/>
     </row>
     <row r="120" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A120" s="6"/>
-      <c r="B120" s="6"/>
-      <c r="C120" s="7"/>
-      <c r="D120" s="7"/>
-      <c r="E120" s="1"/>
-      <c r="F120" s="5"/>
-      <c r="G120" s="5"/>
-      <c r="H120" s="1"/>
-      <c r="I120" s="1"/>
+      <c r="A120" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B120" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C120" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="D120" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E120" s="1">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="F120" s="5">
+        <v>8</v>
+      </c>
+      <c r="G120" s="5">
+        <v>6</v>
+      </c>
+      <c r="H120" s="1">
+        <v>7</v>
+      </c>
+      <c r="I120" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="J120" s="1"/>
-      <c r="K120" s="9"/>
+      <c r="K120" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
       <c r="L120" s="1"/>
       <c r="M120" s="1"/>
       <c r="N120" s="1"/>

</xml_diff>

<commit_message>
new data et meilleure importation data selon , ou ;
</commit_message>
<xml_diff>
--- a/data/spike.xlsx
+++ b/data/spike.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilpe\Documents\DOCUMENTS\ActuRank\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83F537C6-17CC-4637-BBAA-F7288B1B81D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D492EA0-E77A-4675-93C3-73CE7F6A4828}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-1260" yWindow="13120" windowWidth="21600" windowHeight="11270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1136" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1196" uniqueCount="72">
   <si>
     <t>players</t>
   </si>
@@ -249,6 +249,9 @@
   </si>
   <si>
     <t>18/09/2025</t>
+  </si>
+  <si>
+    <t>23/09/2025</t>
   </si>
 </sst>
 </file>
@@ -5881,7 +5884,7 @@
         <v>27</v>
       </c>
       <c r="E132" s="1">
-        <f t="shared" ref="E132:E218" si="4">IF(F132&gt;G132,1,0)</f>
+        <f t="shared" ref="E132:E230" si="4">IF(F132&gt;G132,1,0)</f>
         <v>1</v>
       </c>
       <c r="F132" s="5">
@@ -5898,7 +5901,7 @@
       </c>
       <c r="J132" s="1"/>
       <c r="K132" s="9" t="str">
-        <f t="shared" ref="K132:K195" si="5">IF(OR(OR(AND(OR(A132=B132,A132=C132,A132=D132,B132=C132,B132=D132,C132=D132),OR(A132&lt;&gt;"",D132&lt;&gt;"")),H132&gt;MAX(F132:G132),B132=C132),OR(AND(ISBLANK(A132)=FALSE,ISNA(VLOOKUP(A132,$M$3:$O$27,1,FALSE))),ISNA(VLOOKUP(B132,$M$3:$O$27,1,FALSE)),ISNA(VLOOKUP(C132,$M$3:$O$27,1,FALSE)),AND(ISBLANK(D132)=FALSE,ISNA(VLOOKUP(D132,$M$3:$O$27,1,FALSE))),OR(COUNTBLANK(A132:D132)=1,COUNTBLANK(A132:D132)=3))),"ERREUR","")</f>
+        <f t="shared" ref="K132:K193" si="5">IF(OR(OR(AND(OR(A132=B132,A132=C132,A132=D132,B132=C132,B132=D132,C132=D132),OR(A132&lt;&gt;"",D132&lt;&gt;"")),H132&gt;MAX(F132:G132),B132=C132),OR(AND(ISBLANK(A132)=FALSE,ISNA(VLOOKUP(A132,$M$3:$O$27,1,FALSE))),ISNA(VLOOKUP(B132,$M$3:$O$27,1,FALSE)),ISNA(VLOOKUP(C132,$M$3:$O$27,1,FALSE)),AND(ISBLANK(D132)=FALSE,ISNA(VLOOKUP(D132,$M$3:$O$27,1,FALSE))),OR(COUNTBLANK(A132:D132)=1,COUNTBLANK(A132:D132)=3))),"ERREUR","")</f>
         <v/>
       </c>
       <c r="L132" s="1"/>
@@ -9213,7 +9216,7 @@
       </c>
       <c r="J217" s="1"/>
       <c r="K217" s="9" t="str">
-        <f t="shared" ref="K217:K218" si="8">IF(OR(OR(AND(OR(A217=B217,A217=C217,A217=D217,B217=C217,B217=D217,C217=D217),OR(A217&lt;&gt;"",D217&lt;&gt;"")),H217&gt;MAX(F217:G217),B217=C217),OR(AND(ISBLANK(A217)=FALSE,ISNA(VLOOKUP(A217,$M$3:$O$27,1,FALSE))),ISNA(VLOOKUP(B217,$M$3:$O$27,1,FALSE)),ISNA(VLOOKUP(C217,$M$3:$O$27,1,FALSE)),AND(ISBLANK(D217)=FALSE,ISNA(VLOOKUP(D217,$M$3:$O$27,1,FALSE))),OR(COUNTBLANK(A217:D217)=1,COUNTBLANK(A217:D217)=3))),"ERREUR","")</f>
+        <f t="shared" ref="K217:K222" si="8">IF(OR(OR(AND(OR(A217=B217,A217=C217,A217=D217,B217=C217,B217=D217,C217=D217),OR(A217&lt;&gt;"",D217&lt;&gt;"")),H217&gt;MAX(F217:G217),B217=C217),OR(AND(ISBLANK(A217)=FALSE,ISNA(VLOOKUP(A217,$M$3:$O$27,1,FALSE))),ISNA(VLOOKUP(B217,$M$3:$O$27,1,FALSE)),ISNA(VLOOKUP(C217,$M$3:$O$27,1,FALSE)),AND(ISBLANK(D217)=FALSE,ISNA(VLOOKUP(D217,$M$3:$O$27,1,FALSE))),OR(COUNTBLANK(A217:D217)=1,COUNTBLANK(A217:D217)=3))),"ERREUR","")</f>
         <v/>
       </c>
       <c r="L217" s="1"/>
@@ -9261,83 +9264,190 @@
       <c r="O218" s="1"/>
     </row>
     <row r="219" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A219" s="6"/>
-      <c r="B219" s="6"/>
-      <c r="C219" s="7"/>
-      <c r="D219" s="7"/>
-      <c r="E219" s="1"/>
-      <c r="F219" s="5"/>
-      <c r="G219" s="5"/>
-      <c r="H219" s="1"/>
-      <c r="I219" s="1"/>
+      <c r="A219" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B219" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C219" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D219" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="E219" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F219" s="5">
+        <v>11</v>
+      </c>
+      <c r="G219" s="5">
+        <v>5</v>
+      </c>
+      <c r="H219" s="1">
+        <v>11</v>
+      </c>
+      <c r="I219" s="1" t="s">
+        <v>71</v>
+      </c>
       <c r="J219" s="1"/>
-      <c r="K219" s="9"/>
+      <c r="K219" s="9" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
       <c r="L219" s="1"/>
       <c r="M219" s="1"/>
       <c r="N219" s="1"/>
       <c r="O219" s="1"/>
     </row>
     <row r="220" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A220" s="6"/>
-      <c r="B220" s="6"/>
-      <c r="C220" s="7"/>
-      <c r="D220" s="7"/>
-      <c r="E220" s="1"/>
-      <c r="F220" s="5"/>
-      <c r="G220" s="5"/>
-      <c r="H220" s="1"/>
-      <c r="I220" s="1"/>
+      <c r="A220" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B220" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C220" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D220" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="E220" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F220" s="5">
+        <v>11</v>
+      </c>
+      <c r="G220" s="5">
+        <v>7</v>
+      </c>
+      <c r="H220" s="1">
+        <v>11</v>
+      </c>
+      <c r="I220" s="1" t="s">
+        <v>71</v>
+      </c>
       <c r="J220" s="1"/>
-      <c r="K220" s="9"/>
+      <c r="K220" s="9" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
       <c r="L220" s="1"/>
       <c r="M220" s="1"/>
       <c r="N220" s="1"/>
       <c r="O220" s="1"/>
     </row>
     <row r="221" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A221" s="6"/>
-      <c r="B221" s="6"/>
-      <c r="C221" s="7"/>
-      <c r="D221" s="7"/>
-      <c r="E221" s="1"/>
-      <c r="F221" s="5"/>
-      <c r="G221" s="5"/>
-      <c r="H221" s="1"/>
-      <c r="I221" s="1"/>
+      <c r="A221" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B221" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C221" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D221" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="E221" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F221" s="5">
+        <v>11</v>
+      </c>
+      <c r="G221" s="5">
+        <v>2</v>
+      </c>
+      <c r="H221" s="1">
+        <v>11</v>
+      </c>
+      <c r="I221" s="1" t="s">
+        <v>71</v>
+      </c>
       <c r="J221" s="1"/>
-      <c r="K221" s="9"/>
+      <c r="K221" s="9" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
       <c r="L221" s="1"/>
       <c r="M221" s="1"/>
       <c r="N221" s="1"/>
       <c r="O221" s="1"/>
     </row>
     <row r="222" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A222" s="6"/>
-      <c r="B222" s="6"/>
-      <c r="C222" s="7"/>
-      <c r="D222" s="7"/>
-      <c r="E222" s="1"/>
-      <c r="F222" s="5"/>
-      <c r="G222" s="5"/>
-      <c r="H222" s="1"/>
-      <c r="I222" s="1"/>
+      <c r="A222" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B222" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C222" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D222" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="E222" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F222" s="5">
+        <v>7</v>
+      </c>
+      <c r="G222" s="5">
+        <v>5</v>
+      </c>
+      <c r="H222" s="1">
+        <v>7</v>
+      </c>
+      <c r="I222" s="1" t="s">
+        <v>71</v>
+      </c>
       <c r="J222" s="1"/>
-      <c r="K222" s="9"/>
+      <c r="K222" s="9" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
       <c r="L222" s="1"/>
       <c r="M222" s="1"/>
       <c r="N222" s="1"/>
       <c r="O222" s="1"/>
     </row>
     <row r="223" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A223" s="6"/>
-      <c r="B223" s="6"/>
-      <c r="C223" s="7"/>
-      <c r="D223" s="7"/>
-      <c r="E223" s="1"/>
-      <c r="F223" s="5"/>
-      <c r="G223" s="5"/>
-      <c r="H223" s="1"/>
-      <c r="I223" s="1"/>
+      <c r="A223" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B223" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="C223" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D223" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E223" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F223" s="5">
+        <v>7</v>
+      </c>
+      <c r="G223" s="5">
+        <v>2</v>
+      </c>
+      <c r="H223" s="1">
+        <v>7</v>
+      </c>
+      <c r="I223" s="1" t="s">
+        <v>71</v>
+      </c>
       <c r="J223" s="1"/>
       <c r="K223" s="9"/>
       <c r="L223" s="1"/>
@@ -9346,15 +9456,34 @@
       <c r="O223" s="1"/>
     </row>
     <row r="224" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A224" s="6"/>
-      <c r="B224" s="6"/>
-      <c r="C224" s="7"/>
-      <c r="D224" s="7"/>
-      <c r="E224" s="1"/>
-      <c r="F224" s="5"/>
-      <c r="G224" s="5"/>
-      <c r="H224" s="1"/>
-      <c r="I224" s="1"/>
+      <c r="A224" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B224" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C224" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D224" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="E224" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F224" s="5">
+        <v>8</v>
+      </c>
+      <c r="G224" s="5">
+        <v>6</v>
+      </c>
+      <c r="H224" s="1">
+        <v>7</v>
+      </c>
+      <c r="I224" s="1" t="s">
+        <v>71</v>
+      </c>
       <c r="J224" s="1"/>
       <c r="K224" s="9"/>
       <c r="L224" s="1"/>
@@ -9363,15 +9492,34 @@
       <c r="O224" s="1"/>
     </row>
     <row r="225" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A225" s="6"/>
-      <c r="B225" s="6"/>
-      <c r="C225" s="7"/>
-      <c r="D225" s="7"/>
-      <c r="E225" s="1"/>
-      <c r="F225" s="5"/>
-      <c r="G225" s="5"/>
-      <c r="H225" s="1"/>
-      <c r="I225" s="1"/>
+      <c r="A225" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B225" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C225" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D225" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E225" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F225" s="5">
+        <v>7</v>
+      </c>
+      <c r="G225" s="5">
+        <v>4</v>
+      </c>
+      <c r="H225" s="1">
+        <v>7</v>
+      </c>
+      <c r="I225" s="1" t="s">
+        <v>71</v>
+      </c>
       <c r="J225" s="1"/>
       <c r="K225" s="9"/>
       <c r="L225" s="1"/>
@@ -9380,15 +9528,34 @@
       <c r="O225" s="1"/>
     </row>
     <row r="226" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A226" s="6"/>
-      <c r="B226" s="6"/>
-      <c r="C226" s="7"/>
-      <c r="D226" s="7"/>
-      <c r="E226" s="1"/>
-      <c r="F226" s="5"/>
-      <c r="G226" s="5"/>
-      <c r="H226" s="1"/>
-      <c r="I226" s="1"/>
+      <c r="A226" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B226" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C226" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="D226" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E226" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F226" s="5">
+        <v>7</v>
+      </c>
+      <c r="G226" s="5">
+        <v>5</v>
+      </c>
+      <c r="H226" s="1">
+        <v>7</v>
+      </c>
+      <c r="I226" s="1" t="s">
+        <v>71</v>
+      </c>
       <c r="J226" s="1"/>
       <c r="K226" s="9"/>
       <c r="L226" s="1"/>
@@ -9397,15 +9564,34 @@
       <c r="O226" s="1"/>
     </row>
     <row r="227" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A227" s="6"/>
-      <c r="B227" s="6"/>
-      <c r="C227" s="7"/>
-      <c r="D227" s="7"/>
-      <c r="E227" s="1"/>
-      <c r="F227" s="5"/>
-      <c r="G227" s="5"/>
-      <c r="H227" s="1"/>
-      <c r="I227" s="1"/>
+      <c r="A227" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B227" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C227" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D227" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E227" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F227" s="5">
+        <v>7</v>
+      </c>
+      <c r="G227" s="5">
+        <v>1</v>
+      </c>
+      <c r="H227" s="1">
+        <v>7</v>
+      </c>
+      <c r="I227" s="1" t="s">
+        <v>71</v>
+      </c>
       <c r="J227" s="1"/>
       <c r="K227" s="9"/>
       <c r="L227" s="1"/>
@@ -9414,15 +9600,34 @@
       <c r="O227" s="1"/>
     </row>
     <row r="228" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A228" s="6"/>
-      <c r="B228" s="6"/>
-      <c r="C228" s="7"/>
-      <c r="D228" s="7"/>
-      <c r="E228" s="1"/>
-      <c r="F228" s="5"/>
-      <c r="G228" s="5"/>
-      <c r="H228" s="1"/>
-      <c r="I228" s="1"/>
+      <c r="A228" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B228" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C228" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D228" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="E228" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F228" s="5">
+        <v>7</v>
+      </c>
+      <c r="G228" s="5">
+        <v>2</v>
+      </c>
+      <c r="H228" s="1">
+        <v>7</v>
+      </c>
+      <c r="I228" s="1" t="s">
+        <v>71</v>
+      </c>
       <c r="J228" s="1"/>
       <c r="K228" s="9"/>
       <c r="L228" s="1"/>
@@ -9431,15 +9636,34 @@
       <c r="O228" s="1"/>
     </row>
     <row r="229" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A229" s="6"/>
-      <c r="B229" s="6"/>
-      <c r="C229" s="7"/>
-      <c r="D229" s="7"/>
-      <c r="E229" s="1"/>
-      <c r="F229" s="5"/>
-      <c r="G229" s="5"/>
-      <c r="H229" s="1"/>
-      <c r="I229" s="1"/>
+      <c r="A229" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B229" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C229" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D229" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E229" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F229" s="5">
+        <v>8</v>
+      </c>
+      <c r="G229" s="5">
+        <v>6</v>
+      </c>
+      <c r="H229" s="1">
+        <v>7</v>
+      </c>
+      <c r="I229" s="1" t="s">
+        <v>71</v>
+      </c>
       <c r="J229" s="1"/>
       <c r="K229" s="9"/>
       <c r="L229" s="1"/>
@@ -9448,15 +9672,34 @@
       <c r="O229" s="1"/>
     </row>
     <row r="230" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A230" s="6"/>
-      <c r="B230" s="6"/>
-      <c r="C230" s="7"/>
-      <c r="D230" s="7"/>
-      <c r="E230" s="1"/>
-      <c r="F230" s="5"/>
-      <c r="G230" s="5"/>
-      <c r="H230" s="1"/>
-      <c r="I230" s="1"/>
+      <c r="A230" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B230" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C230" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D230" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E230" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F230" s="5">
+        <v>7</v>
+      </c>
+      <c r="G230" s="5">
+        <v>3</v>
+      </c>
+      <c r="H230" s="1">
+        <v>7</v>
+      </c>
+      <c r="I230" s="1" t="s">
+        <v>71</v>
+      </c>
       <c r="J230" s="1"/>
       <c r="K230" s="9"/>
       <c r="L230" s="1"/>

</xml_diff>

<commit_message>
data mi octobre 2025
</commit_message>
<xml_diff>
--- a/data/spike.xlsx
+++ b/data/spike.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilpe\Documents\DOCUMENTS\ActuRank\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D492EA0-E77A-4675-93C3-73CE7F6A4828}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75BBA88F-1864-4B79-BE2E-2080DD63BADF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-1260" yWindow="13120" windowWidth="21600" windowHeight="11270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9120" yWindow="10800" windowWidth="12980" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1196" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1321" uniqueCount="74">
   <si>
     <t>players</t>
   </si>
@@ -252,6 +252,12 @@
   </si>
   <si>
     <t>23/09/2025</t>
+  </si>
+  <si>
+    <t>14/10/2025</t>
+  </si>
+  <si>
+    <t>15/10/2025</t>
   </si>
 </sst>
 </file>
@@ -5884,7 +5890,7 @@
         <v>27</v>
       </c>
       <c r="E132" s="1">
-        <f t="shared" ref="E132:E230" si="4">IF(F132&gt;G132,1,0)</f>
+        <f t="shared" ref="E132:E255" si="4">IF(F132&gt;G132,1,0)</f>
         <v>1</v>
       </c>
       <c r="F132" s="5">
@@ -8709,7 +8715,7 @@
       </c>
       <c r="J204" s="1"/>
       <c r="K204" s="9" t="str">
-        <f t="shared" ref="K204:K216" si="7">IF(OR(OR(AND(OR(A204=B204,A204=C204,A204=D204,B204=C204,B204=D204,C204=D204),OR(A204&lt;&gt;"",D204&lt;&gt;"")),H204&gt;MAX(F204:G204),B204=C204),OR(AND(ISBLANK(A204)=FALSE,ISNA(VLOOKUP(A204,$M$3:$O$27,1,FALSE))),ISNA(VLOOKUP(B204,$M$3:$O$27,1,FALSE)),ISNA(VLOOKUP(C204,$M$3:$O$27,1,FALSE)),AND(ISBLANK(D204)=FALSE,ISNA(VLOOKUP(D204,$M$3:$O$27,1,FALSE))),OR(COUNTBLANK(A204:D204)=1,COUNTBLANK(A204:D204)=3))),"ERREUR","")</f>
+        <f t="shared" ref="K204:K255" si="7">IF(OR(OR(AND(OR(A204=B204,A204=C204,A204=D204,B204=C204,B204=D204,C204=D204),OR(A204&lt;&gt;"",D204&lt;&gt;"")),H204&gt;MAX(F204:G204),B204=C204),OR(AND(ISBLANK(A204)=FALSE,ISNA(VLOOKUP(A204,$M$3:$O$27,1,FALSE))),ISNA(VLOOKUP(B204,$M$3:$O$27,1,FALSE)),ISNA(VLOOKUP(C204,$M$3:$O$27,1,FALSE)),AND(ISBLANK(D204)=FALSE,ISNA(VLOOKUP(D204,$M$3:$O$27,1,FALSE))),OR(COUNTBLANK(A204:D204)=1,COUNTBLANK(A204:D204)=3))),"ERREUR","")</f>
         <v/>
       </c>
       <c r="L204" s="1"/>
@@ -9216,7 +9222,7 @@
       </c>
       <c r="J217" s="1"/>
       <c r="K217" s="9" t="str">
-        <f t="shared" ref="K217:K222" si="8">IF(OR(OR(AND(OR(A217=B217,A217=C217,A217=D217,B217=C217,B217=D217,C217=D217),OR(A217&lt;&gt;"",D217&lt;&gt;"")),H217&gt;MAX(F217:G217),B217=C217),OR(AND(ISBLANK(A217)=FALSE,ISNA(VLOOKUP(A217,$M$3:$O$27,1,FALSE))),ISNA(VLOOKUP(B217,$M$3:$O$27,1,FALSE)),ISNA(VLOOKUP(C217,$M$3:$O$27,1,FALSE)),AND(ISBLANK(D217)=FALSE,ISNA(VLOOKUP(D217,$M$3:$O$27,1,FALSE))),OR(COUNTBLANK(A217:D217)=1,COUNTBLANK(A217:D217)=3))),"ERREUR","")</f>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="L217" s="1"/>
@@ -9255,7 +9261,7 @@
       </c>
       <c r="J218" s="1"/>
       <c r="K218" s="9" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="L218" s="1"/>
@@ -9294,7 +9300,7 @@
       </c>
       <c r="J219" s="1"/>
       <c r="K219" s="9" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="L219" s="1"/>
@@ -9333,7 +9339,7 @@
       </c>
       <c r="J220" s="1"/>
       <c r="K220" s="9" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="L220" s="1"/>
@@ -9372,7 +9378,7 @@
       </c>
       <c r="J221" s="1"/>
       <c r="K221" s="9" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="L221" s="1"/>
@@ -9411,7 +9417,7 @@
       </c>
       <c r="J222" s="1"/>
       <c r="K222" s="9" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
       <c r="L222" s="1"/>
@@ -9449,7 +9455,10 @@
         <v>71</v>
       </c>
       <c r="J223" s="1"/>
-      <c r="K223" s="9"/>
+      <c r="K223" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L223" s="1"/>
       <c r="M223" s="1"/>
       <c r="N223" s="1"/>
@@ -9485,7 +9494,10 @@
         <v>71</v>
       </c>
       <c r="J224" s="1"/>
-      <c r="K224" s="9"/>
+      <c r="K224" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L224" s="1"/>
       <c r="M224" s="1"/>
       <c r="N224" s="1"/>
@@ -9521,7 +9533,10 @@
         <v>71</v>
       </c>
       <c r="J225" s="1"/>
-      <c r="K225" s="9"/>
+      <c r="K225" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L225" s="1"/>
       <c r="M225" s="1"/>
       <c r="N225" s="1"/>
@@ -9557,7 +9572,10 @@
         <v>71</v>
       </c>
       <c r="J226" s="1"/>
-      <c r="K226" s="9"/>
+      <c r="K226" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L226" s="1"/>
       <c r="M226" s="1"/>
       <c r="N226" s="1"/>
@@ -9593,7 +9611,10 @@
         <v>71</v>
       </c>
       <c r="J227" s="1"/>
-      <c r="K227" s="9"/>
+      <c r="K227" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L227" s="1"/>
       <c r="M227" s="1"/>
       <c r="N227" s="1"/>
@@ -9629,7 +9650,10 @@
         <v>71</v>
       </c>
       <c r="J228" s="1"/>
-      <c r="K228" s="9"/>
+      <c r="K228" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L228" s="1"/>
       <c r="M228" s="1"/>
       <c r="N228" s="1"/>
@@ -9665,7 +9689,10 @@
         <v>71</v>
       </c>
       <c r="J229" s="1"/>
-      <c r="K229" s="9"/>
+      <c r="K229" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L229" s="1"/>
       <c r="M229" s="1"/>
       <c r="N229" s="1"/>
@@ -9701,432 +9728,985 @@
         <v>71</v>
       </c>
       <c r="J230" s="1"/>
-      <c r="K230" s="9"/>
+      <c r="K230" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L230" s="1"/>
       <c r="M230" s="1"/>
       <c r="N230" s="1"/>
       <c r="O230" s="1"/>
     </row>
     <row r="231" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A231" s="6"/>
-      <c r="B231" s="6"/>
-      <c r="C231" s="7"/>
-      <c r="D231" s="7"/>
-      <c r="E231" s="1"/>
-      <c r="F231" s="5"/>
-      <c r="G231" s="5"/>
-      <c r="H231" s="1"/>
-      <c r="I231" s="1"/>
+      <c r="A231" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B231" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C231" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D231" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E231" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F231" s="5">
+        <v>10</v>
+      </c>
+      <c r="G231" s="5">
+        <v>8</v>
+      </c>
+      <c r="H231" s="1">
+        <v>7</v>
+      </c>
+      <c r="I231" s="1" t="s">
+        <v>72</v>
+      </c>
       <c r="J231" s="1"/>
-      <c r="K231" s="9"/>
+      <c r="K231" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L231" s="1"/>
       <c r="M231" s="1"/>
       <c r="N231" s="1"/>
       <c r="O231" s="1"/>
     </row>
     <row r="232" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A232" s="6"/>
-      <c r="B232" s="6"/>
-      <c r="C232" s="7"/>
-      <c r="D232" s="7"/>
-      <c r="E232" s="1"/>
-      <c r="F232" s="5"/>
-      <c r="G232" s="5"/>
-      <c r="H232" s="1"/>
-      <c r="I232" s="1"/>
+      <c r="A232" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B232" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C232" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D232" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E232" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F232" s="5">
+        <v>7</v>
+      </c>
+      <c r="G232" s="5">
+        <v>3</v>
+      </c>
+      <c r="H232" s="1">
+        <v>7</v>
+      </c>
+      <c r="I232" s="1" t="s">
+        <v>72</v>
+      </c>
       <c r="J232" s="1"/>
-      <c r="K232" s="9"/>
+      <c r="K232" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L232" s="1"/>
       <c r="M232" s="1"/>
       <c r="N232" s="1"/>
       <c r="O232" s="1"/>
     </row>
     <row r="233" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A233" s="6"/>
-      <c r="B233" s="6"/>
-      <c r="C233" s="7"/>
-      <c r="D233" s="7"/>
-      <c r="E233" s="1"/>
-      <c r="F233" s="5"/>
-      <c r="G233" s="5"/>
-      <c r="H233" s="1"/>
-      <c r="I233" s="1"/>
+      <c r="A233" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B233" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C233" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D233" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E233" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F233" s="5">
+        <v>7</v>
+      </c>
+      <c r="G233" s="5">
+        <v>3</v>
+      </c>
+      <c r="H233" s="1">
+        <v>7</v>
+      </c>
+      <c r="I233" s="1" t="s">
+        <v>72</v>
+      </c>
       <c r="J233" s="1"/>
-      <c r="K233" s="9"/>
+      <c r="K233" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L233" s="1"/>
       <c r="M233" s="1"/>
       <c r="N233" s="1"/>
       <c r="O233" s="1"/>
     </row>
     <row r="234" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A234" s="6"/>
-      <c r="B234" s="6"/>
-      <c r="C234" s="7"/>
-      <c r="D234" s="7"/>
-      <c r="E234" s="1"/>
-      <c r="F234" s="5"/>
-      <c r="G234" s="5"/>
-      <c r="H234" s="1"/>
-      <c r="I234" s="1"/>
+      <c r="A234" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B234" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C234" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D234" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E234" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F234" s="5">
+        <v>8</v>
+      </c>
+      <c r="G234" s="5">
+        <v>6</v>
+      </c>
+      <c r="H234" s="1">
+        <v>7</v>
+      </c>
+      <c r="I234" s="1" t="s">
+        <v>72</v>
+      </c>
       <c r="J234" s="1"/>
-      <c r="K234" s="9"/>
+      <c r="K234" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L234" s="1"/>
       <c r="M234" s="1"/>
       <c r="N234" s="1"/>
       <c r="O234" s="1"/>
     </row>
     <row r="235" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A235" s="6"/>
-      <c r="B235" s="6"/>
-      <c r="C235" s="7"/>
-      <c r="D235" s="7"/>
-      <c r="E235" s="1"/>
-      <c r="F235" s="5"/>
-      <c r="G235" s="5"/>
-      <c r="H235" s="1"/>
-      <c r="I235" s="1"/>
+      <c r="A235" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B235" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C235" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D235" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E235" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F235" s="5">
+        <v>8</v>
+      </c>
+      <c r="G235" s="5">
+        <v>6</v>
+      </c>
+      <c r="H235" s="1">
+        <v>7</v>
+      </c>
+      <c r="I235" s="1" t="s">
+        <v>72</v>
+      </c>
       <c r="J235" s="1"/>
-      <c r="K235" s="9"/>
+      <c r="K235" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L235" s="1"/>
       <c r="M235" s="1"/>
       <c r="N235" s="1"/>
       <c r="O235" s="1"/>
     </row>
     <row r="236" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A236" s="6"/>
-      <c r="B236" s="6"/>
-      <c r="C236" s="7"/>
-      <c r="D236" s="7"/>
-      <c r="E236" s="1"/>
-      <c r="F236" s="5"/>
-      <c r="G236" s="5"/>
-      <c r="H236" s="1"/>
-      <c r="I236" s="1"/>
+      <c r="A236" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B236" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C236" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D236" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E236" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F236" s="5">
+        <v>7</v>
+      </c>
+      <c r="G236" s="5">
+        <v>5</v>
+      </c>
+      <c r="H236" s="1">
+        <v>7</v>
+      </c>
+      <c r="I236" s="1" t="s">
+        <v>72</v>
+      </c>
       <c r="J236" s="1"/>
-      <c r="K236" s="9"/>
+      <c r="K236" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L236" s="1"/>
       <c r="M236" s="1"/>
       <c r="N236" s="1"/>
       <c r="O236" s="1"/>
     </row>
     <row r="237" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A237" s="6"/>
-      <c r="B237" s="6"/>
-      <c r="C237" s="7"/>
-      <c r="D237" s="7"/>
-      <c r="E237" s="1"/>
-      <c r="F237" s="5"/>
-      <c r="G237" s="5"/>
-      <c r="H237" s="1"/>
-      <c r="I237" s="1"/>
+      <c r="A237" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B237" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C237" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D237" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E237" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F237" s="5">
+        <v>7</v>
+      </c>
+      <c r="G237" s="5">
+        <v>5</v>
+      </c>
+      <c r="H237" s="1">
+        <v>7</v>
+      </c>
+      <c r="I237" s="1" t="s">
+        <v>72</v>
+      </c>
       <c r="J237" s="1"/>
-      <c r="K237" s="9"/>
+      <c r="K237" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L237" s="1"/>
       <c r="M237" s="1"/>
       <c r="N237" s="1"/>
       <c r="O237" s="1"/>
     </row>
     <row r="238" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A238" s="6"/>
-      <c r="B238" s="6"/>
-      <c r="C238" s="7"/>
-      <c r="D238" s="7"/>
-      <c r="E238" s="1"/>
-      <c r="F238" s="5"/>
-      <c r="G238" s="5"/>
-      <c r="H238" s="1"/>
-      <c r="I238" s="1"/>
+      <c r="A238" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B238" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C238" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D238" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E238" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F238" s="5">
+        <v>11</v>
+      </c>
+      <c r="G238" s="5">
+        <v>8</v>
+      </c>
+      <c r="H238" s="1">
+        <v>11</v>
+      </c>
+      <c r="I238" s="1" t="s">
+        <v>72</v>
+      </c>
       <c r="J238" s="1"/>
-      <c r="K238" s="9"/>
+      <c r="K238" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L238" s="1"/>
       <c r="M238" s="1"/>
       <c r="N238" s="1"/>
       <c r="O238" s="1"/>
     </row>
     <row r="239" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A239" s="6"/>
-      <c r="B239" s="6"/>
-      <c r="C239" s="7"/>
-      <c r="D239" s="7"/>
-      <c r="E239" s="1"/>
-      <c r="F239" s="5"/>
-      <c r="G239" s="5"/>
-      <c r="H239" s="1"/>
-      <c r="I239" s="1"/>
+      <c r="A239" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B239" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C239" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D239" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E239" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F239" s="5">
+        <v>7</v>
+      </c>
+      <c r="G239" s="5">
+        <v>4</v>
+      </c>
+      <c r="H239" s="1">
+        <v>7</v>
+      </c>
+      <c r="I239" s="1" t="s">
+        <v>72</v>
+      </c>
       <c r="J239" s="1"/>
-      <c r="K239" s="9"/>
+      <c r="K239" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L239" s="1"/>
       <c r="M239" s="1"/>
       <c r="N239" s="1"/>
       <c r="O239" s="1"/>
     </row>
     <row r="240" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A240" s="6"/>
-      <c r="B240" s="6"/>
-      <c r="C240" s="7"/>
-      <c r="D240" s="7"/>
-      <c r="E240" s="1"/>
-      <c r="F240" s="5"/>
-      <c r="G240" s="5"/>
-      <c r="H240" s="1"/>
-      <c r="I240" s="1"/>
+      <c r="A240" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B240" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C240" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D240" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E240" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F240" s="5">
+        <v>9</v>
+      </c>
+      <c r="G240" s="5">
+        <v>7</v>
+      </c>
+      <c r="H240" s="1">
+        <v>7</v>
+      </c>
+      <c r="I240" s="1" t="s">
+        <v>72</v>
+      </c>
       <c r="J240" s="1"/>
-      <c r="K240" s="9"/>
+      <c r="K240" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L240" s="1"/>
       <c r="M240" s="1"/>
       <c r="N240" s="1"/>
       <c r="O240" s="1"/>
     </row>
     <row r="241" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A241" s="6"/>
-      <c r="B241" s="6"/>
-      <c r="C241" s="7"/>
-      <c r="D241" s="7"/>
-      <c r="E241" s="1"/>
-      <c r="F241" s="5"/>
-      <c r="G241" s="5"/>
-      <c r="H241" s="1"/>
-      <c r="I241" s="1"/>
+      <c r="A241" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B241" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C241" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D241" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E241" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F241" s="5">
+        <v>13</v>
+      </c>
+      <c r="G241" s="5">
+        <v>8</v>
+      </c>
+      <c r="H241" s="1">
+        <v>13</v>
+      </c>
+      <c r="I241" s="1" t="s">
+        <v>72</v>
+      </c>
       <c r="J241" s="1"/>
-      <c r="K241" s="9"/>
+      <c r="K241" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L241" s="1"/>
       <c r="M241" s="1"/>
       <c r="N241" s="1"/>
       <c r="O241" s="1"/>
     </row>
     <row r="242" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A242" s="6"/>
-      <c r="B242" s="6"/>
-      <c r="C242" s="7"/>
-      <c r="D242" s="7"/>
-      <c r="E242" s="1"/>
-      <c r="F242" s="5"/>
-      <c r="G242" s="5"/>
-      <c r="H242" s="1"/>
-      <c r="I242" s="1"/>
+      <c r="A242" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B242" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C242" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D242" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="E242" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F242" s="5">
+        <v>7</v>
+      </c>
+      <c r="G242" s="5">
+        <v>5</v>
+      </c>
+      <c r="H242" s="1">
+        <v>7</v>
+      </c>
+      <c r="I242" s="1" t="s">
+        <v>72</v>
+      </c>
       <c r="J242" s="1"/>
-      <c r="K242" s="9"/>
+      <c r="K242" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L242" s="1"/>
       <c r="M242" s="1"/>
       <c r="N242" s="1"/>
       <c r="O242" s="1"/>
     </row>
     <row r="243" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A243" s="6"/>
-      <c r="B243" s="6"/>
-      <c r="C243" s="7"/>
-      <c r="D243" s="7"/>
-      <c r="E243" s="1"/>
-      <c r="F243" s="5"/>
-      <c r="G243" s="5"/>
-      <c r="H243" s="1"/>
-      <c r="I243" s="1"/>
+      <c r="A243" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B243" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C243" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D243" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E243" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F243" s="5">
+        <v>8</v>
+      </c>
+      <c r="G243" s="5">
+        <v>6</v>
+      </c>
+      <c r="H243" s="1">
+        <v>7</v>
+      </c>
+      <c r="I243" s="1" t="s">
+        <v>72</v>
+      </c>
       <c r="J243" s="1"/>
-      <c r="K243" s="9"/>
+      <c r="K243" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L243" s="1"/>
       <c r="M243" s="1"/>
       <c r="N243" s="1"/>
       <c r="O243" s="1"/>
     </row>
     <row r="244" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A244" s="6"/>
-      <c r="B244" s="6"/>
-      <c r="C244" s="7"/>
-      <c r="D244" s="7"/>
-      <c r="E244" s="1"/>
-      <c r="F244" s="5"/>
-      <c r="G244" s="5"/>
-      <c r="H244" s="1"/>
-      <c r="I244" s="1"/>
+      <c r="A244" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B244" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C244" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D244" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E244" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F244" s="5">
+        <v>7</v>
+      </c>
+      <c r="G244" s="5">
+        <v>4</v>
+      </c>
+      <c r="H244" s="1">
+        <v>7</v>
+      </c>
+      <c r="I244" s="1" t="s">
+        <v>72</v>
+      </c>
       <c r="J244" s="1"/>
-      <c r="K244" s="9"/>
+      <c r="K244" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L244" s="1"/>
       <c r="M244" s="1"/>
       <c r="N244" s="1"/>
       <c r="O244" s="1"/>
     </row>
     <row r="245" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A245" s="6"/>
-      <c r="B245" s="6"/>
-      <c r="C245" s="7"/>
-      <c r="D245" s="7"/>
-      <c r="E245" s="1"/>
-      <c r="F245" s="5"/>
-      <c r="G245" s="5"/>
-      <c r="H245" s="1"/>
-      <c r="I245" s="1"/>
+      <c r="A245" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B245" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C245" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="D245" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E245" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F245" s="5">
+        <v>10</v>
+      </c>
+      <c r="G245" s="5">
+        <v>8</v>
+      </c>
+      <c r="H245" s="1">
+        <v>7</v>
+      </c>
+      <c r="I245" s="1" t="s">
+        <v>72</v>
+      </c>
       <c r="J245" s="1"/>
-      <c r="K245" s="9"/>
+      <c r="K245" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L245" s="1"/>
       <c r="M245" s="1"/>
       <c r="N245" s="1"/>
       <c r="O245" s="1"/>
     </row>
     <row r="246" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A246" s="6"/>
-      <c r="B246" s="6"/>
-      <c r="C246" s="7"/>
-      <c r="D246" s="7"/>
-      <c r="E246" s="1"/>
-      <c r="F246" s="5"/>
-      <c r="G246" s="5"/>
-      <c r="H246" s="1"/>
-      <c r="I246" s="1"/>
+      <c r="A246" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B246" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C246" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D246" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E246" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F246" s="5">
+        <v>8</v>
+      </c>
+      <c r="G246" s="5">
+        <v>6</v>
+      </c>
+      <c r="H246" s="1">
+        <v>7</v>
+      </c>
+      <c r="I246" s="1" t="s">
+        <v>72</v>
+      </c>
       <c r="J246" s="1"/>
-      <c r="K246" s="9"/>
+      <c r="K246" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L246" s="1"/>
       <c r="M246" s="1"/>
       <c r="N246" s="1"/>
       <c r="O246" s="1"/>
     </row>
     <row r="247" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A247" s="6"/>
-      <c r="B247" s="6"/>
-      <c r="C247" s="7"/>
-      <c r="D247" s="7"/>
-      <c r="E247" s="1"/>
-      <c r="F247" s="5"/>
-      <c r="G247" s="5"/>
-      <c r="H247" s="1"/>
-      <c r="I247" s="1"/>
+      <c r="A247" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B247" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C247" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D247" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E247" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F247" s="5">
+        <v>11</v>
+      </c>
+      <c r="G247" s="5">
+        <v>8</v>
+      </c>
+      <c r="H247" s="1">
+        <v>11</v>
+      </c>
+      <c r="I247" s="1" t="s">
+        <v>73</v>
+      </c>
       <c r="J247" s="1"/>
-      <c r="K247" s="9"/>
+      <c r="K247" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L247" s="1"/>
       <c r="M247" s="1"/>
       <c r="N247" s="1"/>
       <c r="O247" s="1"/>
     </row>
     <row r="248" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A248" s="6"/>
-      <c r="B248" s="6"/>
-      <c r="C248" s="7"/>
-      <c r="D248" s="7"/>
-      <c r="E248" s="1"/>
-      <c r="F248" s="5"/>
-      <c r="G248" s="5"/>
-      <c r="H248" s="1"/>
-      <c r="I248" s="1"/>
+      <c r="A248" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B248" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C248" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D248" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E248" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F248" s="5">
+        <v>11</v>
+      </c>
+      <c r="G248" s="5">
+        <v>6</v>
+      </c>
+      <c r="H248" s="1">
+        <v>11</v>
+      </c>
+      <c r="I248" s="1" t="s">
+        <v>73</v>
+      </c>
       <c r="J248" s="1"/>
-      <c r="K248" s="9"/>
+      <c r="K248" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L248" s="1"/>
       <c r="M248" s="1"/>
       <c r="N248" s="1"/>
       <c r="O248" s="1"/>
     </row>
     <row r="249" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A249" s="6"/>
-      <c r="B249" s="6"/>
-      <c r="C249" s="7"/>
-      <c r="D249" s="7"/>
-      <c r="E249" s="1"/>
-      <c r="F249" s="5"/>
-      <c r="G249" s="5"/>
-      <c r="H249" s="1"/>
-      <c r="I249" s="1"/>
+      <c r="A249" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B249" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C249" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D249" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E249" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F249" s="5">
+        <v>11</v>
+      </c>
+      <c r="G249" s="5">
+        <v>8</v>
+      </c>
+      <c r="H249" s="1">
+        <v>11</v>
+      </c>
+      <c r="I249" s="1" t="s">
+        <v>73</v>
+      </c>
       <c r="J249" s="1"/>
-      <c r="K249" s="9"/>
+      <c r="K249" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L249" s="1"/>
       <c r="M249" s="1"/>
       <c r="N249" s="1"/>
       <c r="O249" s="1"/>
     </row>
     <row r="250" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A250" s="6"/>
-      <c r="B250" s="6"/>
-      <c r="C250" s="7"/>
-      <c r="D250" s="7"/>
-      <c r="E250" s="1"/>
-      <c r="F250" s="5"/>
-      <c r="G250" s="5"/>
-      <c r="H250" s="1"/>
-      <c r="I250" s="1"/>
+      <c r="A250" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B250" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C250" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D250" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E250" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F250" s="5">
+        <v>11</v>
+      </c>
+      <c r="G250" s="5">
+        <v>9</v>
+      </c>
+      <c r="H250" s="1">
+        <v>11</v>
+      </c>
+      <c r="I250" s="1" t="s">
+        <v>73</v>
+      </c>
       <c r="J250" s="1"/>
-      <c r="K250" s="9"/>
+      <c r="K250" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L250" s="1"/>
       <c r="M250" s="1"/>
       <c r="N250" s="1"/>
       <c r="O250" s="1"/>
     </row>
     <row r="251" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A251" s="6"/>
-      <c r="B251" s="6"/>
-      <c r="C251" s="7"/>
-      <c r="D251" s="7"/>
-      <c r="E251" s="1"/>
-      <c r="F251" s="5"/>
-      <c r="G251" s="5"/>
-      <c r="H251" s="1"/>
-      <c r="I251" s="1"/>
+      <c r="A251" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B251" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C251" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D251" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E251" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F251" s="5">
+        <v>11</v>
+      </c>
+      <c r="G251" s="5">
+        <v>9</v>
+      </c>
+      <c r="H251" s="1">
+        <v>11</v>
+      </c>
+      <c r="I251" s="1" t="s">
+        <v>73</v>
+      </c>
       <c r="J251" s="1"/>
-      <c r="K251" s="9"/>
+      <c r="K251" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L251" s="1"/>
       <c r="M251" s="1"/>
       <c r="N251" s="1"/>
       <c r="O251" s="1"/>
     </row>
     <row r="252" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A252" s="6"/>
-      <c r="B252" s="6"/>
-      <c r="C252" s="7"/>
-      <c r="D252" s="7"/>
-      <c r="E252" s="1"/>
-      <c r="F252" s="5"/>
-      <c r="G252" s="5"/>
-      <c r="H252" s="1"/>
-      <c r="I252" s="1"/>
+      <c r="A252" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B252" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C252" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D252" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E252" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F252" s="5">
+        <v>11</v>
+      </c>
+      <c r="G252" s="5">
+        <v>5</v>
+      </c>
+      <c r="H252" s="1">
+        <v>11</v>
+      </c>
+      <c r="I252" s="1" t="s">
+        <v>73</v>
+      </c>
       <c r="J252" s="1"/>
-      <c r="K252" s="9"/>
+      <c r="K252" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L252" s="1"/>
       <c r="M252" s="1"/>
       <c r="N252" s="1"/>
       <c r="O252" s="1"/>
     </row>
     <row r="253" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A253" s="6"/>
-      <c r="B253" s="6"/>
-      <c r="C253" s="7"/>
-      <c r="D253" s="7"/>
-      <c r="E253" s="1"/>
-      <c r="F253" s="5"/>
-      <c r="G253" s="5"/>
-      <c r="H253" s="1"/>
-      <c r="I253" s="1"/>
+      <c r="A253" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B253" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C253" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D253" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E253" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F253" s="5">
+        <v>11</v>
+      </c>
+      <c r="G253" s="5">
+        <v>9</v>
+      </c>
+      <c r="H253" s="1">
+        <v>11</v>
+      </c>
+      <c r="I253" s="1" t="s">
+        <v>73</v>
+      </c>
       <c r="J253" s="1"/>
-      <c r="K253" s="9"/>
+      <c r="K253" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L253" s="1"/>
       <c r="M253" s="1"/>
       <c r="N253" s="1"/>
       <c r="O253" s="1"/>
     </row>
     <row r="254" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A254" s="6"/>
-      <c r="B254" s="6"/>
-      <c r="C254" s="7"/>
-      <c r="D254" s="7"/>
-      <c r="E254" s="1"/>
-      <c r="F254" s="5"/>
-      <c r="G254" s="5"/>
-      <c r="H254" s="1"/>
-      <c r="I254" s="1"/>
+      <c r="A254" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B254" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C254" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D254" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E254" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F254" s="5">
+        <v>11</v>
+      </c>
+      <c r="G254" s="5">
+        <v>7</v>
+      </c>
+      <c r="H254" s="1">
+        <v>11</v>
+      </c>
+      <c r="I254" s="1" t="s">
+        <v>73</v>
+      </c>
       <c r="J254" s="1"/>
-      <c r="K254" s="9"/>
+      <c r="K254" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L254" s="1"/>
       <c r="M254" s="1"/>
       <c r="N254" s="1"/>
       <c r="O254" s="1"/>
     </row>
     <row r="255" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A255" s="6"/>
-      <c r="B255" s="6"/>
-      <c r="C255" s="7"/>
-      <c r="D255" s="7"/>
-      <c r="E255" s="1"/>
-      <c r="F255" s="5"/>
-      <c r="G255" s="5"/>
-      <c r="H255" s="1"/>
-      <c r="I255" s="1"/>
+      <c r="A255" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B255" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C255" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D255" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E255" s="1">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="F255" s="5">
+        <v>13</v>
+      </c>
+      <c r="G255" s="5">
+        <v>11</v>
+      </c>
+      <c r="H255" s="1">
+        <v>13</v>
+      </c>
+      <c r="I255" s="1" t="s">
+        <v>73</v>
+      </c>
       <c r="J255" s="1"/>
-      <c r="K255" s="9"/>
+      <c r="K255" s="9" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
       <c r="L255" s="1"/>
       <c r="M255" s="1"/>
       <c r="N255" s="1"/>

</xml_diff>